<commit_message>
Correct reviewed model semantics, dimensions and backend conditions
</commit_message>
<xml_diff>
--- a/dist/downloads/model-documents/kimi-k1.5.xlsx
+++ b/dist/downloads/model-documents/kimi-k1.5.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="算子表" sheetId="1" r:id="R8cb0be50bd284e5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型参数" sheetId="2" r:id="Rac27ec3d07184705"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="算子表" sheetId="1" r:id="R0b66261e9cd2434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型参数" sheetId="2" r:id="R994adfd69c7446a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3469,7 +3469,7 @@
         </x:is>
       </x:c>
       <x:c r="C7" s="24" t="str">
-        <x:f>IF(ISNUMBER(C6),IF(AND(C20&gt;=1,MOD(C6,C20)=0),C6/C20,"未核验"),"未核验")</x:f>
+        <x:f>IF(ISNUMBER(C20),IF(C20&gt;=1,IF(MOD(C20,1)=0,IF(ISNUMBER(C6),IF(MOD(C6,C20)=0,C6/C20,"未核验"),"未核验"),"未核验"),"未核验"),"未核验")</x:f>
         <x:v>未核验</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
@@ -3733,7 +3733,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D20" s="24"/>
-      <x:c r="E20" s="24"/>
+      <x:c r="E20" s="24" t="str">
+        <x:f>IF(ISNUMBER(C20),IF(C20&gt;=1,IF(MOD(C20,1)=0,"正整数场景输入；实际支持未核验","须为正整数"),"须为正整数"),"须为正整数")</x:f>
+        <x:v>正整数场景输入；实际支持未核验</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="24" t="str">
@@ -3746,7 +3749,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="D21" s="24"/>
-      <x:c r="E21" s="24"/>
+      <x:c r="E21" s="24" t="str">
+        <x:f>IF(ISNUMBER(C21),IF(C21&gt;=1,IF(MOD(C21,1)=0,"正整数场景输入；实际支持未核验","须为正整数"),"须为正整数"),"须为正整数")</x:f>
+        <x:v>正整数场景输入；实际支持未核验</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="24" t="str">
@@ -3881,8 +3887,8 @@
       <x:c r="E33" s="24"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
-    <x:dataValidation type="whole" operator="between" sqref="C3:C4">
+  <x:dataValidations count="3">
+    <x:dataValidation type="whole" operator="between" sqref="C3">
       <x:formula1>1</x:formula1>
       <x:formula2>16</x:formula2>
     </x:dataValidation>
@@ -3890,6 +3896,9 @@
       <x:formula1>1</x:formula1>
       <x:formula2>8</x:formula2>
     </x:dataValidation>
+    <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C20:C21">
+      <x:formula1>1</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>